<commit_message>
Remove the owner's name from the example show, the brief and the workbook
The Designer field is left blank. The workbook was edited inside its XML only,
so formulas, formatting and cached results are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference/The_Ballroom_Array_Weights_v6.xlsx
+++ b/reference/The_Ballroom_Array_Weights_v6.xlsx
@@ -84,7 +84,7 @@
     <t xml:space="preserve">Designer</t>
   </si>
   <si>
-    <t xml:space="preserve">Mark Hughes</t>
+    <t xml:space="preserve"/>
   </si>
   <si>
     <t xml:space="preserve">Load over people?</t>
@@ -5895,7 +5895,7 @@
       <c r="F7" s="48"/>
       <c r="G7" s="47" t="str">
         <f aca="false">IF(Calc!B3="","",Calc!B3)</f>
-        <v>Mark Hughes</v>
+        <v/>
       </c>
       <c r="H7" s="47"/>
     </row>

</xml_diff>